<commit_message>
Modify the web UI and few errors
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_29274321_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_29274321_table1_v1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT17"/>
+  <dimension ref="A1:AV13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,87 +564,97 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>P-value note</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>BP(Position)</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>RA 1(Reported Allele 1)</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>RA 2(Reported Allele 2)</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Note on alleles and AF</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>ReportedAF(MAF)</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>AFincases</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>AFincontrols</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Effect Size Type (OR or Beta)</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>EffectSize(altvsref)</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>95%ConfidenceInterval</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Confirmed affected genes, causal variants, evidence</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Genome build (hg18/hg37/hg38)</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Pubmed PMID</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>PMCID</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Table Ref in paper</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Table links</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>LocusName</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -710,10 +720,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N2" t="n">
+        <v>757</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
@@ -728,13 +736,21 @@
           <t>European ancestry</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>dfsajklfdsaf</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>dsafa</t>
+        </is>
+      </c>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
@@ -744,61 +760,55 @@
         </is>
       </c>
       <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
+      <c r="AB2" t="n">
+        <v>8</v>
       </c>
       <c r="AC2" t="n">
         <v>2.54e-08</v>
       </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>20647323.0</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="n">
+        <v>20647323</v>
+      </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>0.16</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="n">
+        <v>0.16</v>
+      </c>
       <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr">
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL2" t="n">
+      <c r="AM2" t="n">
         <v>0.41</v>
       </c>
-      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr">
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>GFRA2, LZTS1</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -862,10 +872,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N3" t="n">
+        <v>757</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
@@ -880,7 +888,11 @@
           <t>European ancestry</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>dasfsd</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
           <t>Group</t>
@@ -896,61 +908,55 @@
         </is>
       </c>
       <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
+      <c r="AB3" t="n">
+        <v>12</v>
       </c>
       <c r="AC3" t="n">
         <v>2.53e-08</v>
       </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>13870464.0</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="n">
+        <v>13870464</v>
+      </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
       <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr">
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL3" t="n">
+      <c r="AM3" t="n">
         <v>-1.02</v>
       </c>
-      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr">
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS3" t="inlineStr">
+      <c r="AT3" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t>GRIN2B</t>
         </is>
       </c>
+      <c r="AV3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1014,10 +1020,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N4" t="n">
+        <v>757</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
@@ -1048,66 +1052,60 @@
         </is>
       </c>
       <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>17.0</t>
-        </is>
+      <c r="AB4" t="n">
+        <v>17</v>
       </c>
       <c r="AC4" t="n">
         <v>2.03e-08</v>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>59687842.0</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="n">
+        <v>59687842</v>
+      </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>0.44</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="n">
+        <v>0.44</v>
+      </c>
       <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr">
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL4" t="n">
+      <c r="AM4" t="n">
         <v>-0.53</v>
       </c>
-      <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr">
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS4" t="inlineStr">
+      <c r="AT4" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr">
+      <c r="AU4" t="inlineStr">
         <is>
           <t>BRIP1, NACA2</t>
         </is>
       </c>
+      <c r="AV4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rs2378873</t>
+          <t>rs10775009</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1166,10 +1164,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N5" t="n">
+        <v>757</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
@@ -1196,66 +1192,64 @@
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>rs2378873</t>
+          <t>rs10775009</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>17.0</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>59687842.0</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AB5" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1.59e-09</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="n">
+        <v>119390525</v>
+      </c>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>0.44</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="n">
+        <v>0.34</v>
+      </c>
       <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr">
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
+      <c r="AM5" t="n">
+        <v>0.51</v>
+      </c>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr">
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS5" t="inlineStr">
+      <c r="AT5" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>BRIP1, NACA2</t>
-        </is>
-      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>SRRM4</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rs10775009</t>
+          <t>rs2819438</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1314,10 +1308,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N6" t="n">
+        <v>757</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -1344,70 +1336,64 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>rs10775009</t>
+          <t>rs2819438</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
+      <c r="AB6" t="n">
+        <v>14</v>
       </c>
       <c r="AC6" t="n">
-        <v>1.59e-09</v>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>119390525.0</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
+        <v>6.94e-09</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="n">
+        <v>105385352</v>
+      </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>0.34</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="n">
+        <v>0.13</v>
+      </c>
       <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr">
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL6" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AM6" t="inlineStr"/>
+      <c r="AM6" t="n">
+        <v>-0.8</v>
+      </c>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr">
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS6" t="inlineStr">
+      <c r="AT6" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT6" t="inlineStr">
-        <is>
-          <t>SRRM4</t>
-        </is>
-      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>PLD4, C14orf79</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rs2819438</t>
+          <t>rs4921790</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1466,10 +1452,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N7" t="n">
+        <v>757</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -1496,70 +1480,64 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>rs2819438</t>
+          <t>rs4921790</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>14.0</t>
-        </is>
+      <c r="AB7" t="n">
+        <v>8</v>
       </c>
       <c r="AC7" t="n">
-        <v>6.94e-09</v>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>105385352.0</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr"/>
+        <v>4.58e-09</v>
+      </c>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="n">
+        <v>17496561</v>
+      </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>0.13</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr">
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL7" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="AM7" t="inlineStr"/>
+      <c r="AM7" t="n">
+        <v>0.61</v>
+      </c>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr">
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
+      <c r="AT7" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>PLD4, C14orf79</t>
-        </is>
-      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>PDGFRL, MTUS1</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rs2819438</t>
+          <t>rs74834332</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1618,10 +1596,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N8" t="n">
+        <v>757</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -1648,66 +1624,64 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>rs2819438</t>
+          <t>rs74834332</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>14.0</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>105385352.0</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AB8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>4.3e-08</v>
+      </c>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="n">
+        <v>57739164</v>
+      </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>0.13</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="n">
+        <v>0.03</v>
+      </c>
       <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr">
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
+      <c r="AM8" t="n">
+        <v>0.79</v>
+      </c>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr">
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS8" t="inlineStr">
+      <c r="AT8" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT8" t="inlineStr">
-        <is>
-          <t>PLD4, C14orf79</t>
-        </is>
-      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>DAB1</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rs4921790</t>
+          <t>rs12268753</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1766,10 +1740,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N9" t="n">
+        <v>757</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
@@ -1796,70 +1768,64 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>rs4921790</t>
+          <t>rs12268753</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
+      <c r="AB9" t="n">
+        <v>10</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.58e-09</v>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>17496561.0</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
+        <v>2.01e-08</v>
+      </c>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="n">
+        <v>53818149</v>
+      </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="n">
+        <v>0.21</v>
+      </c>
       <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr">
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL9" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="AM9" t="inlineStr"/>
+      <c r="AM9" t="n">
+        <v>0.3</v>
+      </c>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr">
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS9" t="inlineStr">
+      <c r="AT9" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>PDGFRL, MTUS1</t>
-        </is>
-      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>PRKG1</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rs4921790</t>
+          <t>rs111882035</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1918,10 +1884,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N10" t="n">
+        <v>757</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
@@ -1948,66 +1912,64 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>rs4921790</t>
+          <t>rs111882035</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>17496561.0</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr"/>
+      <c r="AB10" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>2.74e-08</v>
+      </c>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="n">
+        <v>86416554</v>
+      </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="AI10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="n">
+        <v>0.02</v>
+      </c>
       <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr">
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AM10" t="n">
+        <v>-0.93</v>
+      </c>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
-      <c r="AP10" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr">
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS10" t="inlineStr">
+      <c r="AT10" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT10" t="inlineStr">
-        <is>
-          <t>PDGFRL, MTUS1</t>
-        </is>
-      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>ARHGAP24</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rs74834332</t>
+          <t>rs73705514</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2066,10 +2028,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N11" t="n">
+        <v>757</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
@@ -2096,70 +2056,64 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>rs74834332</t>
+          <t>rs73705514</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="AB11" t="n">
+        <v>7</v>
       </c>
       <c r="AC11" t="n">
-        <v>4.3e-08</v>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>57739164.0</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr"/>
+        <v>2.86e-09</v>
+      </c>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="n">
+        <v>88406552</v>
+      </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="AI11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="n">
+        <v>0.02</v>
+      </c>
       <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr">
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL11" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="AM11" t="inlineStr"/>
+      <c r="AM11" t="n">
+        <v>-0.84</v>
+      </c>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
-      <c r="AP11" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ11" t="inlineStr"/>
-      <c r="AR11" t="inlineStr">
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS11" t="inlineStr">
+      <c r="AT11" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT11" t="inlineStr">
-        <is>
-          <t>DAB1</t>
-        </is>
-      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>ZNF804B</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rs12268753</t>
+          <t>rs118130881</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2218,10 +2172,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N12" t="n">
+        <v>757</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
@@ -2248,70 +2200,64 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>rs12268753</t>
+          <t>rs118130881</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
+      <c r="AB12" t="n">
+        <v>8</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.01e-08</v>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>53818149.0</t>
-        </is>
-      </c>
-      <c r="AE12" t="inlineStr"/>
+        <v>1.72e-08</v>
+      </c>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="n">
+        <v>31228770</v>
+      </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr">
-        <is>
-          <t>0.21</t>
-        </is>
-      </c>
-      <c r="AI12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="n">
+        <v>0.04</v>
+      </c>
       <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr">
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AM12" t="inlineStr"/>
+      <c r="AM12" t="n">
+        <v>-0.61</v>
+      </c>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr">
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS12" t="inlineStr">
+      <c r="AT12" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT12" t="inlineStr">
-        <is>
-          <t>PRKG1</t>
-        </is>
-      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>NRG1</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rs111882035</t>
+          <t>rs79846291</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2370,10 +2316,8 @@
           <t>ADNI</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
+      <c r="N13" t="n">
+        <v>757</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -2400,669 +2344,59 @@
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>rs111882035</t>
+          <t>rs79846291</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
+      <c r="AB13" t="n">
+        <v>6</v>
       </c>
       <c r="AC13" t="n">
-        <v>2.74e-08</v>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>86416554.0</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr"/>
+        <v>1.76e-08</v>
+      </c>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="n">
+        <v>136077929</v>
+      </c>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="AI13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="n">
+        <v>0.02</v>
+      </c>
       <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr">
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL13" t="n">
-        <v>-0.93</v>
-      </c>
-      <c r="AM13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr">
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="n">
+        <v>29274321</v>
+      </c>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="AS13" t="inlineStr">
+      <c r="AT13" t="inlineStr">
         <is>
           <t>29274321_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT13" t="inlineStr">
-        <is>
-          <t>ARHGAP24</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>rs73705514</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>29274321_table1_R00013</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>29274321_table1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>linear regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>European ancestry</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>rs73705514</t>
-        </is>
-      </c>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="AC14" t="n">
-        <v>2.86e-09</v>
-      </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>88406552.0</t>
-        </is>
-      </c>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr">
-        <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="AL14" t="n">
-        <v>-0.84</v>
-      </c>
-      <c r="AM14" t="inlineStr"/>
-      <c r="AN14" t="inlineStr"/>
-      <c r="AO14" t="inlineStr"/>
-      <c r="AP14" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS14" t="inlineStr">
-        <is>
-          <t>29274321_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT14" t="inlineStr">
-        <is>
-          <t>ZNF804B</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>rs73705514</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>29274321_table1_R00014</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>29274321_table1</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>linear regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>European ancestry</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>rs73705514</t>
-        </is>
-      </c>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>88406552.0</t>
-        </is>
-      </c>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
-      <c r="AN15" t="inlineStr"/>
-      <c r="AO15" t="inlineStr"/>
-      <c r="AP15" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS15" t="inlineStr">
-        <is>
-          <t>29274321_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT15" t="inlineStr">
-        <is>
-          <t>ZNF804B</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>rs118130881</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>29274321_table1_R00015</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>29274321_table1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>linear regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>European ancestry</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>rs118130881</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="AC16" t="n">
-        <v>1.72e-08</v>
-      </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>31228770.0</t>
-        </is>
-      </c>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr">
-        <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="AL16" t="n">
-        <v>-0.61</v>
-      </c>
-      <c r="AM16" t="inlineStr"/>
-      <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS16" t="inlineStr">
-        <is>
-          <t>29274321_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT16" t="inlineStr">
-        <is>
-          <t>NRG1</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>rs79846291</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>29274321_table1_R00016</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>29274321_table1</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>linear regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>757</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>European ancestry</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>rs79846291</t>
-        </is>
-      </c>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="AC17" t="n">
-        <v>1.76e-08</v>
-      </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>136077929.0</t>
-        </is>
-      </c>
-      <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr"/>
-      <c r="AH17" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr">
-        <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="AL17" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="AM17" t="inlineStr"/>
-      <c r="AN17" t="inlineStr"/>
-      <c r="AO17" t="inlineStr"/>
-      <c r="AP17" t="inlineStr">
-        <is>
-          <t>29274321</t>
-        </is>
-      </c>
-      <c r="AQ17" t="inlineStr"/>
-      <c r="AR17" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS17" t="inlineStr">
-        <is>
-          <t>29274321_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT17" t="inlineStr">
+      <c r="AU13" t="inlineStr">
         <is>
           <t>LINC00271, PDE7B</t>
         </is>
       </c>
+      <c r="AV13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>